<commit_message>
changes made after review
</commit_message>
<xml_diff>
--- a/app/pipeline_output/AKME/mapping_AKME_COMBINED.xlsx
+++ b/app/pipeline_output/AKME/mapping_AKME_COMBINED.xlsx
@@ -12,8 +12,8 @@
     <sheet name="For Review" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Field Mapping'!$A$1:$I$48</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'For Review'!$A$1:$I$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Field Mapping'!$A$1:$I$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'For Review'!$A$1:$I$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I48"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -2334,7 +2334,7 @@
         </is>
       </c>
       <c r="F41" s="3" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.95</v>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
@@ -2343,7 +2343,7 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>The partner field 'LoanTypeName' semantically corresponds to the internal field 'APPLICANTLOANTYPE' which represents the loan type.</t>
+          <t>The field 'LoanTypeName' semantically corresponds to 'APPLICANTLOANTYPE' which represents the type of the loan.</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
@@ -2355,12 +2355,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>Address</t>
+          <t>AddressOR</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>LeadReference</t>
+          <t>LeadAddress</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2370,16 +2370,16 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>BUSINESSVERIFICATIONADDRESS</t>
+          <t>ADDRESSREMARKS</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>loanAccount.customer.verifications.0.address</t>
-        </is>
-      </c>
-      <c r="F42" s="3" t="n">
-        <v>0.93</v>
+          <t>loanAccount.customer.customerAdditional.addressRemarks</t>
+        </is>
+      </c>
+      <c r="F42" s="4" t="n">
+        <v>0.88</v>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>The field 'Address' in the context of 'LeadReference' maps well to the address of a verification or reference person.</t>
+          <t>The field name 'AddressOR' suggests it could be an alternative address or remarks related to an address.</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -2400,12 +2400,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>Relation</t>
+          <t>Remark</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>LeadReference</t>
+          <t>LeadContact</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2415,16 +2415,16 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>BUSINESSVERIFICATIONENTERPRISERELATION1TYPE</t>
+          <t>APPLICANTPERSONALDISCUSSIONCOMMENTS</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>loanAccount.customer.verifications.0.relationship</t>
-        </is>
-      </c>
-      <c r="F43" s="3" t="n">
-        <v>0.9399999999999999</v>
+          <t>loanAccount.customer.personalDiscussionComments</t>
+        </is>
+      </c>
+      <c r="F43" s="4" t="n">
+        <v>0.89</v>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
@@ -2433,7 +2433,7 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>The field 'Relation' in the context of 'LeadReference' maps directly to the relationship type of a verification contact.</t>
+          <t>'Remark' is a general comments field, and 'Personal Discussion Comments' is a suitable specific field for applicant-related remarks.</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
@@ -2445,12 +2445,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>NoOfYearResiding</t>
+          <t>Address</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>LeadAddress</t>
+          <t>LeadReference</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2460,16 +2460,16 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>APPLICANTINCURRENTADDRESSSINCE</t>
+          <t>BUSINESSVERIFICATIONADDRESS</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>loanAccount.customer.inCurrentAddressSince</t>
+          <t>loanAccount.customer.verifications.0.address</t>
         </is>
       </c>
       <c r="F44" s="3" t="n">
-        <v>0.93</v>
+        <v>0.95</v>
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
@@ -2478,7 +2478,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>'Number of Years Residing' is semantically equivalent to the duration since the 'inCurrentAddressSince' date.</t>
+          <t>Given the context of 'LeadReference', this field represents the address of the reference, which matches 'BUSINESSVERIFICATIONADDRESS'.</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr">
@@ -2490,12 +2490,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>OtherName</t>
+          <t>Relation</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>LeadDocument</t>
+          <t>LeadReference</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -2505,25 +2505,25 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
-          <t>DOCUMENTNAME3</t>
+          <t>BUSINESSVERIFICATIONENTERPRISERELATION1TYPE</t>
         </is>
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>loanAccount.loanDocuments.2.document</t>
+          <t>loanAccount.customer.verifications.0.relationship</t>
         </is>
       </c>
       <c r="F45" s="3" t="n">
-        <v>0.9</v>
+        <v>0.96</v>
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>llm_pattern_document_name</t>
+          <t>llm_semantic</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>The column category 'LeadDocument' indicates this field is a document name, even though the field name itself is generic.</t>
+          <t>The field 'Relation' in a 'LeadReference' context clearly maps to the relationship of the reference to the applicant.</t>
         </is>
       </c>
       <c r="I45" s="2" t="inlineStr">
@@ -2535,40 +2535,40 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>DocumentType</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>LeadDocument</t>
+          <t>LeadFinancial</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>DOCUMENT</t>
+          <t>APPLICANT</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>DOCUMENTNAME4</t>
+          <t>CUSTOMERBANKACCOUNTTYPE</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>loanAccount.loanDocuments.3.document</t>
-        </is>
-      </c>
-      <c r="F46" s="3" t="n">
-        <v>0.9</v>
+          <t>loanAccount.customer.customerBankAccounts.0.accountType</t>
+        </is>
+      </c>
+      <c r="F46" s="4" t="n">
+        <v>0.88</v>
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>llm_pattern_document_name</t>
+          <t>llm_semantic</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Contains document keyword 'Document' and no locator keyword.</t>
+          <t>In the 'LeadFinancial' context, 'Type' most likely refers to the bank account type.</t>
         </is>
       </c>
       <c r="I46" s="2" t="inlineStr">
@@ -2580,27 +2580,27 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>FileName</t>
+          <t>TypeName</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>LeadDocument</t>
+          <t>LeadProfile</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>DOCUMENT</t>
+          <t>APPLICANT</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
         <is>
-          <t>DOCUMENTNAME5</t>
+          <t>APPLICANTCUSTOMERTYPE</t>
         </is>
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>loanAccount.loanDocuments.4.document</t>
+          <t>loanAccount.customer.customerType</t>
         </is>
       </c>
       <c r="F47" s="3" t="n">
@@ -2608,12 +2608,12 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>llm_pattern_document_name</t>
+          <t>llm_semantic</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>Contains document keyword 'File' and no locator keyword.</t>
+          <t>In the 'LeadProfile' context, 'TypeName' most likely refers to the customer or applicant type.</t>
         </is>
       </c>
       <c r="I47" s="2" t="inlineStr">
@@ -2625,50 +2625,275 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
+          <t>FatherSpouse</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>LeadProfile</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>APPLICANT</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>APPLICANTFATHERNAME</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>loanAccount.customer.fatherFirstName</t>
+        </is>
+      </c>
+      <c r="F48" s="4" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>llm_semantic</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>The field seems to hold either the father's or spouse's name; mapping to father's name as a primary relative.</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>NoOfYearResiding</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>LeadAddress</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>APPLICANT</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>APPLICANTINCURRENTADDRESSSINCE</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>loanAccount.customer.inCurrentAddressSince</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>llm_semantic</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>'Number of years residing' is semantically equivalent to the concept of 'in current address since'.</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>OtherName</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>LeadDocument</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>APPLICANT</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>DOCUMENTNAME3</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>loanAccount.loanDocuments.2.document</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>llm_pattern_document_name</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>The field 'OtherName' in the 'LeadDocument' category indicates the name of a document.</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>DocumentType</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>LeadDocument</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>DOCUMENT</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>DOCUMENTNAME4</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>loanAccount.loanDocuments.3.document</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>llm_pattern_document_name</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>The field 'DocumentType' specifies the type of a document and matches the DOCUMENTNAME pattern.</t>
+        </is>
+      </c>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>FileName</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>LeadDocument</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>DOCUMENT</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>DOCUMENTNAME5</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>loanAccount.loanDocuments.4.document</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>llm_pattern_document_name</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>The field 'FileName' specifies the name of a document file and matches the DOCUMENTNAME pattern.</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
           <t>FilePath</t>
         </is>
       </c>
-      <c r="B48" s="2" t="inlineStr">
+      <c r="B53" s="2" t="inlineStr">
         <is>
           <t>LeadDocument</t>
         </is>
       </c>
-      <c r="C48" s="2" t="inlineStr">
+      <c r="C53" s="2" t="inlineStr">
         <is>
           <t>DOCUMENT</t>
         </is>
       </c>
-      <c r="D48" s="2" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>DOCUMENTID6</t>
         </is>
       </c>
-      <c r="E48" s="2" t="inlineStr">
+      <c r="E53" s="2" t="inlineStr">
         <is>
           <t>loanAccount.loanDocuments.5.documentId</t>
         </is>
       </c>
-      <c r="F48" s="3" t="n">
+      <c r="F53" s="3" t="n">
         <v>0.9</v>
       </c>
-      <c r="G48" s="2" t="inlineStr">
+      <c r="G53" s="2" t="inlineStr">
         <is>
           <t>llm_pattern_document_id</t>
         </is>
       </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>Contains document keyword 'File' and locator keyword 'Path'.</t>
-        </is>
-      </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="H53" s="2" t="inlineStr">
+        <is>
+          <t>The field 'FilePath' contains document and locator keywords ('File', 'Path'), matching the DOCUMENTID pattern.</t>
+        </is>
+      </c>
+      <c r="I53" s="2" t="inlineStr">
         <is>
           <t>NO</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I48"/>
+  <autoFilter ref="A1:I53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2679,7 +2904,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2720,7 +2945,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-04-06 11:50:56</t>
+          <t>2026-04-06 14:59:22</t>
         </is>
       </c>
     </row>
@@ -2741,7 +2966,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7">
@@ -2751,7 +2976,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="9">
@@ -2854,11 +3079,11 @@
     <row r="19">
       <c r="B19" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="20">
@@ -2888,7 +3113,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24">
@@ -2945,7 +3170,7 @@
         </is>
       </c>
       <c r="B30" s="7" t="n">
-        <v>73</v>
+        <v>68</v>
       </c>
     </row>
     <row r="31">
@@ -3198,54 +3423,64 @@
     <row r="52">
       <c r="C52" t="inlineStr">
         <is>
-          <t>... and 53 more</t>
+          <t>... and 48 more</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
+          <t>Mandatory Fields Missing:</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
           <t>Confidence Distribution:</t>
         </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>0.90-1.00</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>0.80-0.89</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="57">
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>0.70-0.79</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>73</v>
       </c>
     </row>
     <row r="58">
       <c r="B58" t="inlineStr">
         <is>
+          <t>0.90-1.00</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>0.80-0.89</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>0.70-0.79</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="B61" t="inlineStr">
+        <is>
           <t>0.00-0.69</t>
         </is>
       </c>
-      <c r="C58" t="n">
+      <c r="C61" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3260,7 +3495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I74"/>
+  <dimension ref="A1:I69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -5709,7 +5944,7 @@
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>AddressOR</t>
+          <t>AddressID</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
@@ -5724,12 +5959,12 @@
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM1</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM1</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F55" s="9" t="n">
@@ -5737,12 +5972,12 @@
       </c>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H55" s="8" t="inlineStr">
         <is>
-          <t>The field 'AddressOR' is ambiguous and does not match any specific address-related excel_key.</t>
+          <t>No specific field for an address identifier exists, so using a general applicant parameter is the correct fallback.</t>
         </is>
       </c>
       <c r="I55" s="8" t="inlineStr">
@@ -5754,12 +5989,12 @@
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>Remark</t>
+          <t>RelationOther</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>LeadContact</t>
+          <t>LeadReference</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
@@ -5769,12 +6004,12 @@
       </c>
       <c r="D56" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM2</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM2</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F56" s="9" t="n">
@@ -5782,12 +6017,12 @@
       </c>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr">
         <is>
-          <t>The generic field 'Remark' in a contact context does not map to a specific applicant remark field.</t>
+          <t>No specific field for an 'other' relationship type exists, so a general applicant parameter is used.</t>
         </is>
       </c>
       <c r="I56" s="8" t="inlineStr">
@@ -5799,12 +6034,12 @@
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
         <is>
-          <t>AddressID</t>
+          <t>CurrentMarketValue</t>
         </is>
       </c>
       <c r="B57" s="8" t="inlineStr">
         <is>
-          <t>LeadAddress</t>
+          <t>LeadLoan</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
@@ -5814,12 +6049,12 @@
       </c>
       <c r="D57" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM3</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E57" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM3</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F57" s="9" t="n">
@@ -5827,12 +6062,12 @@
       </c>
       <c r="G57" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H57" s="8" t="inlineStr">
         <is>
-          <t>There is no specific internal field for a partner's internal 'AddressID'.</t>
+          <t>There is no available field for current market value of an asset, so a general applicant parameter is the correct fallback.</t>
         </is>
       </c>
       <c r="I57" s="8" t="inlineStr">
@@ -5844,12 +6079,12 @@
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>RelationOther</t>
+          <t>TenureType</t>
         </is>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>LeadReference</t>
+          <t>LeadLoan</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
@@ -5859,12 +6094,12 @@
       </c>
       <c r="D58" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM4</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM4</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F58" s="9" t="n">
@@ -5872,12 +6107,12 @@
       </c>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H58" s="8" t="inlineStr">
         <is>
-          <t>There is no specific internal field for a free-text 'Other' relationship for a reference.</t>
+          <t>No available field for tenure type exists, so using a general applicant parameter is the correct fallback.</t>
         </is>
       </c>
       <c r="I58" s="8" t="inlineStr">
@@ -5889,12 +6124,12 @@
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>CurrentMarketValue</t>
+          <t>CibilGenerated</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>LeadLoan</t>
+          <t>LeadProfile</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
@@ -5904,12 +6139,12 @@
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM5</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM5</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F59" s="9" t="n">
@@ -5917,12 +6152,12 @@
       </c>
       <c r="G59" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H59" s="8" t="inlineStr">
         <is>
-          <t>This is a loan-specific attribute not available in the general APPLICANT entity scope.</t>
+          <t>No field exists for a flag indicating CIBIL report generation, so a general applicant parameter is used.</t>
         </is>
       </c>
       <c r="I59" s="8" t="inlineStr">
@@ -5934,12 +6169,12 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>TenureType</t>
+          <t>IsPrimaryText</t>
         </is>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>LeadLoan</t>
+          <t>LeadAddress</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
@@ -5949,12 +6184,12 @@
       </c>
       <c r="D60" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM6</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM6</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F60" s="9" t="n">
@@ -5962,12 +6197,12 @@
       </c>
       <c r="G60" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr">
         <is>
-          <t>This is a loan-specific attribute not available in the general APPLICANT entity scope.</t>
+          <t>No specific field for a primary address indicator exists, so a general applicant parameter is used.</t>
         </is>
       </c>
       <c r="I60" s="8" t="inlineStr">
@@ -5979,12 +6214,12 @@
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>AreaOther</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>LeadFinancial</t>
+          <t>LeadAddress</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
@@ -5994,12 +6229,12 @@
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM7</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM7</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F61" s="9" t="n">
@@ -6007,12 +6242,12 @@
       </c>
       <c r="G61" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H61" s="8" t="inlineStr">
         <is>
-          <t>The field name 'Type' is too generic to be mapped to a specific financial attribute of the applicant.</t>
+          <t>This is a custom free-text field for an address area which does not have a standard equivalent.</t>
         </is>
       </c>
       <c r="I61" s="8" t="inlineStr">
@@ -6024,12 +6259,12 @@
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
         <is>
-          <t>TypeName</t>
+          <t>AreaPanchayatPopulation</t>
         </is>
       </c>
       <c r="B62" s="8" t="inlineStr">
         <is>
-          <t>LeadProfile</t>
+          <t>LeadAddress</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
@@ -6039,12 +6274,12 @@
       </c>
       <c r="D62" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM8</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E62" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM8</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F62" s="9" t="n">
@@ -6052,12 +6287,12 @@
       </c>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H62" s="8" t="inlineStr">
         <is>
-          <t>The field name 'TypeName' is too generic to be mapped to a specific profile attribute of the applicant.</t>
+          <t>This is a highly specific field with no standard equivalent in the available keys.</t>
         </is>
       </c>
       <c r="I62" s="8" t="inlineStr">
@@ -6069,12 +6304,12 @@
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>FatherSpouse</t>
+          <t>IsPrimary</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
         <is>
-          <t>LeadProfile</t>
+          <t>LeadContact</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
@@ -6084,12 +6319,12 @@
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM9</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM9</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F63" s="9" t="n">
@@ -6097,12 +6332,12 @@
       </c>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H63" s="8" t="inlineStr">
         <is>
-          <t>The system uses separate fields for Father Name and Spouse Name; a combined field cannot be mapped.</t>
+          <t>No specific field for a primary contact indicator exists, so a general applicant parameter is used.</t>
         </is>
       </c>
       <c r="I63" s="8" t="inlineStr">
@@ -6114,12 +6349,12 @@
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>CibilGenerated</t>
+          <t>ContactType</t>
         </is>
       </c>
       <c r="B64" s="8" t="inlineStr">
         <is>
-          <t>LeadProfile</t>
+          <t>LeadContact</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
@@ -6129,12 +6364,12 @@
       </c>
       <c r="D64" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM10</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM10</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F64" s="9" t="n">
@@ -6142,12 +6377,12 @@
       </c>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H64" s="8" t="inlineStr">
         <is>
-          <t>There is no specific field to store a CIBIL generation flag or date for an applicant.</t>
+          <t>No specific field for contact type exists, so a general applicant parameter is used.</t>
         </is>
       </c>
       <c r="I64" s="8" t="inlineStr">
@@ -6159,12 +6394,12 @@
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
         <is>
-          <t>IsPrimaryText</t>
+          <t>Value</t>
         </is>
       </c>
       <c r="B65" s="8" t="inlineStr">
         <is>
-          <t>LeadAddress</t>
+          <t>LeadContact</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
@@ -6174,12 +6409,12 @@
       </c>
       <c r="D65" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM11</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E65" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM11</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F65" s="9" t="n">
@@ -6187,12 +6422,12 @@
       </c>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H65" s="8" t="inlineStr">
         <is>
-          <t>There is no specific field for a text representation of a primary address flag.</t>
+          <t>The field 'Value' is too generic in the 'LeadContact' context to map confidently; it could be a phone number or email.</t>
         </is>
       </c>
       <c r="I65" s="8" t="inlineStr">
@@ -6204,12 +6439,12 @@
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>AreaOther</t>
+          <t>Extension</t>
         </is>
       </c>
       <c r="B66" s="8" t="inlineStr">
         <is>
-          <t>LeadAddress</t>
+          <t>LeadContact</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
@@ -6219,12 +6454,12 @@
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM12</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM12</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F66" s="9" t="n">
@@ -6232,12 +6467,12 @@
       </c>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H66" s="8" t="inlineStr">
         <is>
-          <t>There is no specific address field for 'AreaOther'.</t>
+          <t>No specific field for a phone extension exists.</t>
         </is>
       </c>
       <c r="I66" s="8" t="inlineStr">
@@ -6249,12 +6484,12 @@
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
         <is>
-          <t>AreaPanchayatPopulation</t>
+          <t>ReferenceID</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>LeadAddress</t>
+          <t>LeadReference</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
@@ -6264,12 +6499,12 @@
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM13</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM13</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F67" s="9" t="n">
@@ -6277,12 +6512,12 @@
       </c>
       <c r="G67" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H67" s="8" t="inlineStr">
         <is>
-          <t>There is no specific field to store the population of the applicant's area or panchayat.</t>
+          <t>No field for a partner-provided reference ID exists, so a general applicant parameter is used.</t>
         </is>
       </c>
       <c r="I67" s="8" t="inlineStr">
@@ -6294,12 +6529,12 @@
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
         <is>
-          <t>IsPrimary</t>
+          <t>ExShowroomPrice</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>LeadContact</t>
+          <t>LeadLoan</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
@@ -6309,12 +6544,12 @@
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM14</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM14</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F68" s="9" t="n">
@@ -6322,12 +6557,12 @@
       </c>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H68" s="8" t="inlineStr">
         <is>
-          <t>The available contact fields do not have a corresponding 'IsPrimary' flag.</t>
+          <t>No specific field for ex-showroom price is available, so a general applicant parameter is used as a fallback.</t>
         </is>
       </c>
       <c r="I68" s="8" t="inlineStr">
@@ -6339,12 +6574,12 @@
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
         <is>
-          <t>ContactType</t>
+          <t>Details</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>LeadContact</t>
+          <t>LeadBankDetails</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
@@ -6354,12 +6589,12 @@
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM15</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>CUSTOMERPARAM15</t>
+          <t>LOANAPPLICANTPARAM</t>
         </is>
       </c>
       <c r="F69" s="9" t="n">
@@ -6367,12 +6602,12 @@
       </c>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t>llm_customerparameter</t>
+          <t>llm_loanapplicantparam</t>
         </is>
       </c>
       <c r="H69" s="8" t="inlineStr">
         <is>
-          <t>The internal model has dedicated fields for each contact type (mobile, email) rather than a generic 'ContactType' field.</t>
+          <t>'Details' in a bank context is too generic to map to a specific field like account number or branch.</t>
         </is>
       </c>
       <c r="I69" s="8" t="inlineStr">
@@ -6381,233 +6616,8 @@
         </is>
       </c>
     </row>
-    <row r="70">
-      <c r="A70" s="8" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="B70" s="8" t="inlineStr">
-        <is>
-          <t>LeadContact</t>
-        </is>
-      </c>
-      <c r="C70" s="8" t="inlineStr">
-        <is>
-          <t>APPLICANT</t>
-        </is>
-      </c>
-      <c r="D70" s="8" t="inlineStr">
-        <is>
-          <t>CUSTOMERPARAM16</t>
-        </is>
-      </c>
-      <c r="E70" s="8" t="inlineStr">
-        <is>
-          <t>CUSTOMERPARAM16</t>
-        </is>
-      </c>
-      <c r="F70" s="9" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="G70" s="8" t="inlineStr">
-        <is>
-          <t>llm_customerparameter</t>
-        </is>
-      </c>
-      <c r="H70" s="8" t="inlineStr">
-        <is>
-          <t>The generic field 'Value' for a contact cannot be mapped without knowing the contact type.</t>
-        </is>
-      </c>
-      <c r="I70" s="8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="8" t="inlineStr">
-        <is>
-          <t>Extension</t>
-        </is>
-      </c>
-      <c r="B71" s="8" t="inlineStr">
-        <is>
-          <t>LeadContact</t>
-        </is>
-      </c>
-      <c r="C71" s="8" t="inlineStr">
-        <is>
-          <t>APPLICANT</t>
-        </is>
-      </c>
-      <c r="D71" s="8" t="inlineStr">
-        <is>
-          <t>CUSTOMERPARAM17</t>
-        </is>
-      </c>
-      <c r="E71" s="8" t="inlineStr">
-        <is>
-          <t>CUSTOMERPARAM17</t>
-        </is>
-      </c>
-      <c r="F71" s="9" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="G71" s="8" t="inlineStr">
-        <is>
-          <t>llm_customerparameter</t>
-        </is>
-      </c>
-      <c r="H71" s="8" t="inlineStr">
-        <is>
-          <t>There is no specific field for a phone number extension.</t>
-        </is>
-      </c>
-      <c r="I71" s="8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="8" t="inlineStr">
-        <is>
-          <t>ReferenceID</t>
-        </is>
-      </c>
-      <c r="B72" s="8" t="inlineStr">
-        <is>
-          <t>LeadReference</t>
-        </is>
-      </c>
-      <c r="C72" s="8" t="inlineStr">
-        <is>
-          <t>APPLICANT</t>
-        </is>
-      </c>
-      <c r="D72" s="8" t="inlineStr">
-        <is>
-          <t>CUSTOMERPARAM18</t>
-        </is>
-      </c>
-      <c r="E72" s="8" t="inlineStr">
-        <is>
-          <t>CUSTOMERPARAM18</t>
-        </is>
-      </c>
-      <c r="F72" s="9" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="G72" s="8" t="inlineStr">
-        <is>
-          <t>llm_customerparameter</t>
-        </is>
-      </c>
-      <c r="H72" s="8" t="inlineStr">
-        <is>
-          <t>There is no specific internal field for a partner's internal 'ReferenceID'.</t>
-        </is>
-      </c>
-      <c r="I72" s="8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="8" t="inlineStr">
-        <is>
-          <t>ExShowroomPrice</t>
-        </is>
-      </c>
-      <c r="B73" s="8" t="inlineStr">
-        <is>
-          <t>LeadLoan</t>
-        </is>
-      </c>
-      <c r="C73" s="8" t="inlineStr">
-        <is>
-          <t>APPLICANT</t>
-        </is>
-      </c>
-      <c r="D73" s="8" t="inlineStr">
-        <is>
-          <t>CUSTOMERPARAM19</t>
-        </is>
-      </c>
-      <c r="E73" s="8" t="inlineStr">
-        <is>
-          <t>CUSTOMERPARAM19</t>
-        </is>
-      </c>
-      <c r="F73" s="9" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="G73" s="8" t="inlineStr">
-        <is>
-          <t>llm_customerparameter</t>
-        </is>
-      </c>
-      <c r="H73" s="8" t="inlineStr">
-        <is>
-          <t>This vehicle-specific loan attribute is not available in the general APPLICANT entity scope.</t>
-        </is>
-      </c>
-      <c r="I73" s="8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="8" t="inlineStr">
-        <is>
-          <t>Details</t>
-        </is>
-      </c>
-      <c r="B74" s="8" t="inlineStr">
-        <is>
-          <t>LeadBankDetails</t>
-        </is>
-      </c>
-      <c r="C74" s="8" t="inlineStr">
-        <is>
-          <t>APPLICANT</t>
-        </is>
-      </c>
-      <c r="D74" s="8" t="inlineStr">
-        <is>
-          <t>CUSTOMERPARAM20</t>
-        </is>
-      </c>
-      <c r="E74" s="8" t="inlineStr">
-        <is>
-          <t>CUSTOMERPARAM20</t>
-        </is>
-      </c>
-      <c r="F74" s="9" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="G74" s="8" t="inlineStr">
-        <is>
-          <t>llm_customerparameter</t>
-        </is>
-      </c>
-      <c r="H74" s="8" t="inlineStr">
-        <is>
-          <t>The generic term 'Details' in a bank context is too ambiguous to map to a specific field.</t>
-        </is>
-      </c>
-      <c r="I74" s="8" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I74"/>
+  <autoFilter ref="A1:I69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>